<commit_message>
hot fix bao cao nvl
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>DANH SÁCH CÔNG ĐOẠN</t>
   </si>
@@ -51,13 +51,16 @@
   </si>
   <si>
     <t>Mã thống kê</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ngày thứ tự thực hiện </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -79,6 +82,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -116,15 +126,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -410,57 +423,60 @@
   <dimension ref="A1:AMJ2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.140625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="20" style="2" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="13.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" style="2" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" style="2" customWidth="1"/>
-    <col min="13" max="1024" width="9.140625" style="2"/>
+    <col min="1" max="1" width="28.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5703125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" style="1" customWidth="1"/>
+    <col min="13" max="1024" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
     </row>
-    <row r="2" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -468,6 +484,6 @@
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hot fix code process
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -138,6 +138,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -420,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AMJ2"/>
+  <dimension ref="A1:AMJ9"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" style="1" customWidth="1"/>
@@ -438,19 +441,19 @@
     <col min="13" max="1024" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:1024" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
-    <row r="2" spans="1:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1024" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -469,15 +472,19 @@
       <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>9</v>
       </c>
+    </row>
+    <row r="9" spans="1:1024" x14ac:dyDescent="0.25">
+      <c r="AMI9"/>
+      <c r="AMJ9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
hot fix process code
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>DANH SÁCH CÔNG ĐOẠN</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Ngày thứ tự thực hiện </t>
+  </si>
+  <si>
+    <t>Lớp số gộp tồn kho</t>
   </si>
 </sst>
 </file>
@@ -126,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -141,6 +144,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -423,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AMJ9"/>
+  <dimension ref="A1:AMK9"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" style="1" customWidth="1"/>
@@ -433,27 +442,28 @@
     <col min="5" max="5" width="21.5703125" style="1" customWidth="1"/>
     <col min="6" max="6" width="19.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="20" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="17" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5703125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="14.42578125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" style="1" customWidth="1"/>
-    <col min="13" max="1024" width="9.140625" style="1"/>
+    <col min="8" max="9" width="16.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="17" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="1" customWidth="1"/>
+    <col min="14" max="1025" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1024" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:1025" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="7"/>
     </row>
-    <row r="2" spans="1:1024" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1025" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -478,13 +488,16 @@
       <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:1024" x14ac:dyDescent="0.25">
-      <c r="AMI9"/>
+    <row r="9" spans="1:1025" x14ac:dyDescent="0.25">
       <c r="AMJ9"/>
+      <c r="AMK9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
change template process and change logic sync trans am
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportProductProcessTemplate.xlsx
@@ -102,7 +102,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -120,6 +120,26 @@
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -146,10 +166,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -433,25 +453,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AMK9"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="25.5" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="22.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="30.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="31" style="1" customWidth="1"/>
     <col min="6" max="6" width="19.85546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="20" style="1" customWidth="1"/>
-    <col min="8" max="9" width="16.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.28515625" style="1" customWidth="1"/>
     <col min="11" max="11" width="14.5703125" style="1" customWidth="1"/>
     <col min="12" max="12" width="14.42578125" style="1" customWidth="1"/>
     <col min="13" max="13" width="11.7109375" style="1" customWidth="1"/>
     <col min="14" max="1025" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1025" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:1025" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="7"/>
@@ -461,9 +482,10 @@
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
-      <c r="I1" s="6"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
     </row>
-    <row r="2" spans="1:1025" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1025" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -495,13 +517,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:1025" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1025" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="AMJ9"/>
       <c r="AMK9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>